<commit_message>
buscador en el pago
</commit_message>
<xml_diff>
--- a/Empleado.xlsx
+++ b/Empleado.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
   <si>
     <t>Fecha Ingreso</t>
   </si>
@@ -36,6 +36,33 @@
   </si>
   <si>
     <t>Pago</t>
+  </si>
+  <si>
+    <t>2024-10-31 Hora:  20:25</t>
+  </si>
+  <si>
+    <t>eee</t>
+  </si>
+  <si>
+    <t>2024-10-31</t>
+  </si>
+  <si>
+    <t>50000</t>
+  </si>
+  <si>
+    <t>kevin</t>
+  </si>
+  <si>
+    <t>ingeniero</t>
+  </si>
+  <si>
+    <t>fijo</t>
+  </si>
+  <si>
+    <t>caguan</t>
+  </si>
+  <si>
+    <t>1000000</t>
   </si>
 </sst>
 </file>
@@ -80,7 +107,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -109,6 +136,58 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="s">
+        <v>8</v>
+      </c>
+      <c r="B2" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E2" t="s">
+        <v>10</v>
+      </c>
+      <c r="F2" t="s">
+        <v>10</v>
+      </c>
+      <c r="G2" t="s">
+        <v>9</v>
+      </c>
+      <c r="H2" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s">
+        <v>8</v>
+      </c>
+      <c r="B3" t="s">
+        <v>12</v>
+      </c>
+      <c r="C3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" t="s">
+        <v>14</v>
+      </c>
+      <c r="E3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F3" t="s">
+        <v>10</v>
+      </c>
+      <c r="G3" t="s">
+        <v>15</v>
+      </c>
+      <c r="H3" t="s">
+        <v>16</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
puse que se actualice el contador en inventario y pago
</commit_message>
<xml_diff>
--- a/Empleado.xlsx
+++ b/Empleado.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="24" uniqueCount="19">
   <si>
     <t>Fecha Ingreso</t>
   </si>
@@ -38,31 +38,37 @@
     <t>Pago</t>
   </si>
   <si>
-    <t>2024-10-31 Hora:  20:25</t>
-  </si>
-  <si>
-    <t>eee</t>
+    <t>2024-10-31 Hora:  21:54</t>
+  </si>
+  <si>
+    <t>kevin</t>
+  </si>
+  <si>
+    <t>inge</t>
+  </si>
+  <si>
+    <t>fijo</t>
   </si>
   <si>
     <t>2024-10-31</t>
   </si>
   <si>
-    <t>50000</t>
-  </si>
-  <si>
-    <t>kevin</t>
-  </si>
-  <si>
-    <t>ingeniero</t>
-  </si>
-  <si>
-    <t>fijo</t>
-  </si>
-  <si>
     <t>caguan</t>
   </si>
   <si>
-    <t>1000000</t>
+    <t>500000000</t>
+  </si>
+  <si>
+    <t>2024-10-31 Hora:  21:55</t>
+  </si>
+  <si>
+    <t>mancipe</t>
+  </si>
+  <si>
+    <t>medellon</t>
+  </si>
+  <si>
+    <t>5000000</t>
   </si>
 </sst>
 </file>
@@ -144,48 +150,48 @@
         <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="D2" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="E2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G2" t="s">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H2" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>8</v>
+        <v>15</v>
       </c>
       <c r="B3" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="C3" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="E3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F3" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="H3" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
puse el filtro en el empleado"pago"
</commit_message>
<xml_diff>
--- a/Empleado.xlsx
+++ b/Empleado.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="56" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="45">
   <si>
     <t>Fecha Ingreso</t>
   </si>
@@ -47,24 +47,33 @@
     <t>inge</t>
   </si>
   <si>
+    <t>fijoo</t>
+  </si>
+  <si>
+    <t>2024-11-03</t>
+  </si>
+  <si>
+    <t>2024-11-09</t>
+  </si>
+  <si>
+    <t>caguan</t>
+  </si>
+  <si>
+    <t>500000000</t>
+  </si>
+  <si>
+    <t>2024-10-31 Hora:  21:55</t>
+  </si>
+  <si>
+    <t>mancipe</t>
+  </si>
+  <si>
     <t>fijo</t>
   </si>
   <si>
     <t>2024-10-31</t>
   </si>
   <si>
-    <t>caguan</t>
-  </si>
-  <si>
-    <t>500000000</t>
-  </si>
-  <si>
-    <t>2024-10-31 Hora:  21:55</t>
-  </si>
-  <si>
-    <t>mancipe</t>
-  </si>
-  <si>
     <t>medellon</t>
   </si>
   <si>
@@ -117,6 +126,27 @@
   </si>
   <si>
     <t>neiva</t>
+  </si>
+  <si>
+    <t>2024-11-05 Hora:  19:21</t>
+  </si>
+  <si>
+    <t>ingeniero</t>
+  </si>
+  <si>
+    <t>2024-11-05</t>
+  </si>
+  <si>
+    <t>2024-12-05</t>
+  </si>
+  <si>
+    <t>1000000</t>
+  </si>
+  <si>
+    <t>2024-11-05 Hora:  20:09</t>
+  </si>
+  <si>
+    <t>15000000</t>
   </si>
 </sst>
 </file>
@@ -161,7 +191,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:H9"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -207,143 +237,195 @@
         <v>12</v>
       </c>
       <c r="F2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B3" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="C3" t="s">
         <v>10</v>
       </c>
       <c r="D3" t="s">
-        <v>11</v>
+        <v>18</v>
       </c>
       <c r="E3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F3" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="G3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B4" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="D4" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="F4" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="G4" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H4" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="B5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" t="s">
+        <v>24</v>
+      </c>
+      <c r="D5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E5" t="s">
+        <v>26</v>
+      </c>
+      <c r="F5" t="s">
+        <v>33</v>
+      </c>
+      <c r="G5" t="s">
         <v>28</v>
       </c>
-      <c r="C5" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" t="s">
-        <v>29</v>
-      </c>
-      <c r="E5" t="s">
-        <v>23</v>
-      </c>
-      <c r="F5" t="s">
-        <v>30</v>
-      </c>
-      <c r="G5" t="s">
-        <v>25</v>
-      </c>
       <c r="H5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="B6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C6" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+      <c r="F6" t="s">
+        <v>33</v>
+      </c>
+      <c r="G6" t="s">
         <v>28</v>
       </c>
-      <c r="C6" t="s">
-        <v>21</v>
-      </c>
-      <c r="D6" t="s">
-        <v>22</v>
-      </c>
-      <c r="E6" t="s">
-        <v>23</v>
-      </c>
-      <c r="F6" t="s">
-        <v>30</v>
-      </c>
-      <c r="G6" t="s">
-        <v>25</v>
-      </c>
       <c r="H6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
+        <v>36</v>
+      </c>
+      <c r="B7" t="s">
+        <v>31</v>
+      </c>
+      <c r="C7" t="s">
+        <v>24</v>
+      </c>
+      <c r="D7" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" t="s">
+        <v>26</v>
+      </c>
+      <c r="F7" t="s">
         <v>33</v>
       </c>
-      <c r="B7" t="s">
-        <v>28</v>
-      </c>
-      <c r="C7" t="s">
-        <v>21</v>
-      </c>
-      <c r="D7" t="s">
-        <v>22</v>
-      </c>
-      <c r="E7" t="s">
-        <v>23</v>
-      </c>
-      <c r="F7" t="s">
-        <v>30</v>
-      </c>
       <c r="G7" t="s">
+        <v>37</v>
+      </c>
+      <c r="H7" t="s">
         <v>34</v>
       </c>
-      <c r="H7" t="s">
-        <v>31</v>
+    </row>
+    <row r="8">
+      <c r="A8" t="s">
+        <v>38</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8" t="s">
+        <v>39</v>
+      </c>
+      <c r="D8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" t="s">
+        <v>40</v>
+      </c>
+      <c r="F8" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" t="s">
+        <v>14</v>
+      </c>
+      <c r="H8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s">
+        <v>9</v>
+      </c>
+      <c r="C9" t="s">
+        <v>10</v>
+      </c>
+      <c r="D9" t="s">
+        <v>18</v>
+      </c>
+      <c r="E9" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" t="s">
+        <v>14</v>
+      </c>
+      <c r="H9" t="s">
+        <v>44</v>
       </c>
     </row>
   </sheetData>

</xml_diff>